<commit_message>
612 re-doing script network packettracer
</commit_message>
<xml_diff>
--- a/2026-T1/T1B2-ICTNWK612-Plan-manage-troubleshooting-advance/2-tasks/script-PACKETTRACER.xlsx
+++ b/2026-T1/T1B2-ICTNWK612-Plan-manage-troubleshooting-advance/2-tasks/script-PACKETTRACER.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/mannsee/Documents/Assessments/2026-T1/T1B2-ICTNWK612-Plan-manage-troubleshooting-advance/2-tasks/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AC0569FA-17D2-BE43-83F8-76CEC271F9AF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EA0B43C9-A31D-974E-A056-61BFB8D53A63}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="15140" yWindow="680" windowWidth="15120" windowHeight="18980" activeTab="5" xr2:uid="{9C60B164-F6F9-DC45-9E1B-21FD8D75857B}"/>
+    <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="18980" activeTab="7" xr2:uid="{9C60B164-F6F9-DC45-9E1B-21FD8D75857B}"/>
   </bookViews>
   <sheets>
     <sheet name="MS4-3560" sheetId="1" r:id="rId1"/>
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="138" uniqueCount="52">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="58" uniqueCount="17">
   <si>
     <t>enable</t>
   </si>
@@ -68,63 +68,9 @@
     <t>Reload</t>
   </si>
   <si>
-    <t>vlan 10</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> name LAB1</t>
-  </si>
-  <si>
-    <t>interface range fa0/1 - 24</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> switchport mode access</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> switchport access vlan 10</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> spanning-tree portfast</t>
-  </si>
-  <si>
-    <t>interface vlan 10</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> ipv6 address 2001:DB8:10::1/64</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> no shutdown</t>
-  </si>
-  <si>
-    <t>exit</t>
-  </si>
-  <si>
     <t>hostname MS3</t>
   </si>
   <si>
-    <t>vlan 20</t>
-  </si>
-  <si>
-    <t>name LAB2</t>
-  </si>
-  <si>
-    <t>switchport mode access</t>
-  </si>
-  <si>
-    <t>switchport access vlan 20</t>
-  </si>
-  <si>
-    <t>spanning-tree portfast</t>
-  </si>
-  <si>
-    <t>interface vlan 20</t>
-  </si>
-  <si>
-    <t>ipv6 address 2001:DB8:20::1/64</t>
-  </si>
-  <si>
-    <t>no shutdown</t>
-  </si>
-  <si>
     <t>hostname MS2</t>
   </si>
   <si>
@@ -147,57 +93,6 @@
   </si>
   <si>
     <t>show ipv6 general-prefix</t>
-  </si>
-  <si>
-    <t>vlan 30</t>
-  </si>
-  <si>
-    <t>name ADMIN</t>
-  </si>
-  <si>
-    <t>interface range fa0/1 - 20</t>
-  </si>
-  <si>
-    <t>switchport access vlan 30</t>
-  </si>
-  <si>
-    <t>interface vlan 30</t>
-  </si>
-  <si>
-    <t>ipv6 address 2001:DB8:30::1/64</t>
-  </si>
-  <si>
-    <t>vlan 40</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> name ACADEMIC</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> switchport access vlan 40</t>
-  </si>
-  <si>
-    <t>interface vlan 40</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> ipv6 address 2001:DB8:40::1/64</t>
-  </si>
-  <si>
-    <t>vlan 50</t>
-  </si>
-  <si>
-    <t>name SERVER</t>
-  </si>
-  <si>
-    <t>interface range fa0/1 - 12</t>
-  </si>
-  <si>
-    <t>switchport access vlan 50</t>
-  </si>
-  <si>
-    <t>interface vlan 50</t>
-  </si>
-  <si>
-    <t>ipv6 address 2001:DB8:50::1/64</t>
   </si>
 </sst>
 </file>
@@ -227,7 +122,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="4">
     <border>
       <left/>
       <right/>
@@ -235,13 +130,53 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -563,114 +498,53 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A1" t="s">
+      <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A2" t="s">
+      <c r="A2" s="3" t="s">
         <v>1</v>
       </c>
     </row>
     <row r="3" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A3" t="s">
+      <c r="A3" s="3" t="s">
         <v>2</v>
       </c>
     </row>
     <row r="4" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A4" t="s">
+      <c r="A4" s="3" t="s">
         <v>3</v>
       </c>
     </row>
     <row r="5" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A5" t="s">
+      <c r="A5" s="3" t="s">
         <v>4</v>
       </c>
     </row>
     <row r="6" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A6" t="s">
+      <c r="A6" s="3" t="s">
         <v>5</v>
       </c>
     </row>
     <row r="7" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A7" t="s">
+      <c r="A7" s="3" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="8" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A8" t="s">
+      <c r="A8" s="4" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="10" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A10" t="s">
-        <v>0</v>
-      </c>
-    </row>
     <row r="11" spans="1:1" ht="17" x14ac:dyDescent="0.25">
-      <c r="A11" s="1" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="12" spans="1:1" ht="17" x14ac:dyDescent="0.25">
-      <c r="A12" s="1" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="13" spans="1:1" ht="17" x14ac:dyDescent="0.25">
-      <c r="A13" s="1" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="14" spans="1:1" ht="17" x14ac:dyDescent="0.25">
-      <c r="A14" s="1" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="15" spans="1:1" ht="17" x14ac:dyDescent="0.25">
-      <c r="A15" s="1" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="16" spans="1:1" ht="17" x14ac:dyDescent="0.25">
-      <c r="A16" s="1" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="17" spans="1:1" ht="17" x14ac:dyDescent="0.25">
-      <c r="A17" s="1" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="18" spans="1:1" ht="17" x14ac:dyDescent="0.25">
-      <c r="A18" s="1" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="19" spans="1:1" ht="17" x14ac:dyDescent="0.25">
-      <c r="A19" s="1" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="20" spans="1:1" ht="17" x14ac:dyDescent="0.25">
-      <c r="A20" s="1" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="21" spans="1:1" ht="17" x14ac:dyDescent="0.25">
-      <c r="A21" s="1" t="s">
-        <v>17</v>
-      </c>
+      <c r="A11" s="1"/>
     </row>
     <row r="22" spans="1:1" ht="17" x14ac:dyDescent="0.25">
-      <c r="A22" s="1" t="s">
-        <v>17</v>
-      </c>
+      <c r="A22" s="1"/>
     </row>
     <row r="23" spans="1:1" ht="17" x14ac:dyDescent="0.25">
-      <c r="A23" s="1" t="s">
-        <v>6</v>
-      </c>
+      <c r="A23" s="1"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -679,120 +553,50 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{59A2DE29-DDFD-084F-996E-5D8DD645CFD2}">
-  <dimension ref="A1:A28"/>
+  <dimension ref="A1:A8"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="34.1640625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A1" t="s">
+      <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A2" t="s">
+      <c r="A2" s="3" t="s">
         <v>1</v>
       </c>
     </row>
     <row r="3" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A3" t="s">
-        <v>28</v>
+      <c r="A3" s="3" t="s">
+        <v>10</v>
       </c>
     </row>
     <row r="4" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A4" t="s">
+      <c r="A4" s="3" t="s">
         <v>3</v>
       </c>
     </row>
     <row r="5" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A5" t="s">
+      <c r="A5" s="3" t="s">
         <v>4</v>
       </c>
     </row>
     <row r="6" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A6" t="s">
+      <c r="A6" s="3" t="s">
         <v>5</v>
       </c>
     </row>
     <row r="7" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A7" t="s">
+      <c r="A7" s="3" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="8" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A8" t="s">
+      <c r="A8" s="4" t="s">
         <v>7</v>
-      </c>
-    </row>
-    <row r="10" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A10" t="s">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="11" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A11" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="13" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A13" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="14" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A14" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="16" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A16" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="17" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A17" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="18" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A18" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="19" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A19" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="21" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A21" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="22" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A22" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="23" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A23" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="25" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A25" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="26" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A26" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="28" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A28" t="s">
-        <v>6</v>
       </c>
     </row>
   </sheetData>
@@ -802,120 +606,50 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CCC59594-6BB4-1E4A-B489-1D5AC66DAC96}">
-  <dimension ref="A1:A29"/>
+  <dimension ref="A1:A8"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="43.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A1" t="s">
+      <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A2" t="s">
+      <c r="A2" s="3" t="s">
         <v>1</v>
       </c>
     </row>
     <row r="3" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A3" t="s">
-        <v>18</v>
+      <c r="A3" s="3" t="s">
+        <v>8</v>
       </c>
     </row>
     <row r="4" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A4" t="s">
+      <c r="A4" s="3" t="s">
         <v>3</v>
       </c>
     </row>
     <row r="5" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A5" t="s">
+      <c r="A5" s="3" t="s">
         <v>4</v>
       </c>
     </row>
     <row r="6" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A6" t="s">
+      <c r="A6" s="3" t="s">
         <v>5</v>
       </c>
     </row>
     <row r="7" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A7" t="s">
+      <c r="A7" s="3" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="8" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A8" t="s">
+      <c r="A8" s="4" t="s">
         <v>7</v>
-      </c>
-    </row>
-    <row r="11" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A11" t="s">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="12" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A12" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="14" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A14" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="15" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A15" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="17" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A17" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="18" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A18" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="19" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A19" t="s">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="20" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A20" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="22" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A22" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="23" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A23" t="s">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="24" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A24" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="26" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A26" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="27" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A27" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="29" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A29" t="s">
-        <v>6</v>
       </c>
     </row>
   </sheetData>
@@ -925,120 +659,50 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B10D8871-2FF1-AB46-91D6-9529E44202B6}">
-  <dimension ref="A1:A28"/>
+  <dimension ref="A1:A8"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="32.83203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A1" t="s">
+      <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A2" t="s">
+      <c r="A2" s="3" t="s">
         <v>1</v>
       </c>
     </row>
     <row r="3" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A3" t="s">
-        <v>27</v>
+      <c r="A3" s="3" t="s">
+        <v>9</v>
       </c>
     </row>
     <row r="4" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A4" t="s">
+      <c r="A4" s="3" t="s">
         <v>3</v>
       </c>
     </row>
     <row r="5" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A5" t="s">
+      <c r="A5" s="3" t="s">
         <v>4</v>
       </c>
     </row>
     <row r="6" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A6" t="s">
+      <c r="A6" s="3" t="s">
         <v>5</v>
       </c>
     </row>
     <row r="7" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A7" t="s">
+      <c r="A7" s="3" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="8" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A8" t="s">
+      <c r="A8" s="4" t="s">
         <v>7</v>
-      </c>
-    </row>
-    <row r="10" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A10" t="s">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="11" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A11" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="13" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A13" t="s">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="14" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A14" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="16" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A16" t="s">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="17" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A17" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="18" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A18" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="19" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A19" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="21" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A21" t="s">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="22" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A22" t="s">
-        <v>51</v>
-      </c>
-    </row>
-    <row r="23" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A23" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="25" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A25" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="26" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A26" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="28" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A28" t="s">
-        <v>6</v>
       </c>
     </row>
   </sheetData>
@@ -1055,114 +719,83 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A1" t="s">
+      <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A2" t="s">
+      <c r="A2" s="3" t="s">
         <v>1</v>
       </c>
     </row>
     <row r="3" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A3" t="s">
-        <v>29</v>
+      <c r="A3" s="3" t="s">
+        <v>11</v>
       </c>
     </row>
     <row r="4" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A4" t="s">
+      <c r="A4" s="3" t="s">
         <v>3</v>
       </c>
     </row>
     <row r="5" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A5" t="s">
+      <c r="A5" s="3" t="s">
         <v>4</v>
       </c>
     </row>
     <row r="6" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A6" t="s">
+      <c r="A6" s="3" t="s">
         <v>5</v>
       </c>
     </row>
     <row r="7" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A7" t="s">
+      <c r="A7" s="3" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="8" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A8" t="s">
+      <c r="A8" s="4" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="11" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A11" t="s">
-        <v>0</v>
-      </c>
-    </row>
     <row r="12" spans="1:1" ht="17" x14ac:dyDescent="0.25">
-      <c r="A12" s="1" t="s">
-        <v>1</v>
-      </c>
+      <c r="A12" s="1"/>
     </row>
     <row r="14" spans="1:1" ht="17" x14ac:dyDescent="0.25">
-      <c r="A14" s="1" t="s">
-        <v>41</v>
-      </c>
+      <c r="A14" s="1"/>
     </row>
     <row r="15" spans="1:1" ht="17" x14ac:dyDescent="0.25">
-      <c r="A15" s="1" t="s">
-        <v>42</v>
-      </c>
+      <c r="A15" s="1"/>
     </row>
     <row r="17" spans="1:1" ht="17" x14ac:dyDescent="0.25">
-      <c r="A17" s="1" t="s">
-        <v>37</v>
-      </c>
+      <c r="A17" s="1"/>
     </row>
     <row r="18" spans="1:1" ht="17" x14ac:dyDescent="0.25">
-      <c r="A18" s="1" t="s">
-        <v>11</v>
-      </c>
+      <c r="A18" s="1"/>
     </row>
     <row r="19" spans="1:1" ht="17" x14ac:dyDescent="0.25">
-      <c r="A19" s="1" t="s">
-        <v>43</v>
-      </c>
+      <c r="A19" s="1"/>
     </row>
     <row r="20" spans="1:1" ht="17" x14ac:dyDescent="0.25">
-      <c r="A20" s="1" t="s">
-        <v>13</v>
-      </c>
+      <c r="A20" s="1"/>
     </row>
     <row r="22" spans="1:1" ht="17" x14ac:dyDescent="0.25">
-      <c r="A22" s="1" t="s">
-        <v>44</v>
-      </c>
+      <c r="A22" s="1"/>
     </row>
     <row r="23" spans="1:1" ht="17" x14ac:dyDescent="0.25">
-      <c r="A23" s="1" t="s">
-        <v>45</v>
-      </c>
+      <c r="A23" s="1"/>
     </row>
     <row r="24" spans="1:1" ht="17" x14ac:dyDescent="0.25">
-      <c r="A24" s="1" t="s">
-        <v>16</v>
-      </c>
+      <c r="A24" s="1"/>
     </row>
     <row r="26" spans="1:1" ht="17" x14ac:dyDescent="0.25">
-      <c r="A26" s="1" t="s">
-        <v>17</v>
-      </c>
+      <c r="A26" s="1"/>
     </row>
     <row r="27" spans="1:1" ht="17" x14ac:dyDescent="0.25">
-      <c r="A27" s="1" t="s">
-        <v>17</v>
-      </c>
+      <c r="A27" s="1"/>
     </row>
     <row r="29" spans="1:1" ht="17" x14ac:dyDescent="0.25">
-      <c r="A29" s="1" t="s">
-        <v>6</v>
-      </c>
+      <c r="A29" s="1"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -1171,100 +804,50 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6CFEE1F6-6AF7-454F-BBB3-C95B039FA8B6}">
-  <dimension ref="A1:A23"/>
+  <dimension ref="A1:A8"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="36" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A1" t="s">
+      <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A2" t="s">
+      <c r="A2" s="3" t="s">
         <v>1</v>
       </c>
     </row>
     <row r="3" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A3" t="s">
-        <v>30</v>
+      <c r="A3" s="3" t="s">
+        <v>12</v>
       </c>
     </row>
     <row r="4" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A4" t="s">
-        <v>31</v>
+      <c r="A4" s="3" t="s">
+        <v>13</v>
       </c>
     </row>
     <row r="5" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A5" t="s">
+      <c r="A5" s="3" t="s">
         <v>4</v>
       </c>
     </row>
     <row r="6" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A6" t="s">
+      <c r="A6" s="3" t="s">
         <v>5</v>
       </c>
     </row>
     <row r="7" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A7" t="s">
+      <c r="A7" s="3" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="8" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A8" t="s">
+      <c r="A8" s="4" t="s">
         <v>7</v>
-      </c>
-    </row>
-    <row r="11" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A11" t="s">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="12" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A12" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="14" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A14" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="15" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A15" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="16" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A16" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="17" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A17" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="18" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A18" t="s">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="20" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A20" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="21" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A21" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="23" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A23" t="s">
-        <v>6</v>
       </c>
     </row>
   </sheetData>
@@ -1276,44 +859,47 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FD35A78F-566F-7848-A017-7C42AAF25B63}">
   <dimension ref="A1:A8"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="1" max="1" width="46.6640625" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A1" t="s">
+      <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A2" t="s">
+      <c r="A2" s="3" t="s">
         <v>1</v>
       </c>
     </row>
     <row r="3" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A3" t="s">
-        <v>32</v>
+      <c r="A3" s="3" t="s">
+        <v>14</v>
       </c>
     </row>
     <row r="4" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A4" t="s">
-        <v>31</v>
+      <c r="A4" s="3" t="s">
+        <v>13</v>
       </c>
     </row>
     <row r="5" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A5" t="s">
+      <c r="A5" s="3" t="s">
         <v>4</v>
       </c>
     </row>
     <row r="6" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A6" t="s">
+      <c r="A6" s="3" t="s">
         <v>5</v>
       </c>
     </row>
     <row r="7" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A7" t="s">
+      <c r="A7" s="3" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="8" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A8" t="s">
+      <c r="A8" s="4" t="s">
         <v>7</v>
       </c>
     </row>
@@ -1329,12 +915,12 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
-        <v>33</v>
+        <v>15</v>
       </c>
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
-        <v>34</v>
+        <v>16</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
612 implementing VLANs, deleted ipv6 on NON MS0 or MS1
</commit_message>
<xml_diff>
--- a/2026-T1/T1B2-ICTNWK612-Plan-manage-troubleshooting-advance/2-tasks/script-PACKETTRACER.xlsx
+++ b/2026-T1/T1B2-ICTNWK612-Plan-manage-troubleshooting-advance/2-tasks/script-PACKETTRACER.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/mannsee/Documents/Assessments/2026-T1/T1B2-ICTNWK612-Plan-manage-troubleshooting-advance/2-tasks/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EA0B43C9-A31D-974E-A056-61BFB8D53A63}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BB81FEE3-37C1-9241-998F-5F6F7D1ED8D1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="18980" activeTab="7" xr2:uid="{9C60B164-F6F9-DC45-9E1B-21FD8D75857B}"/>
+    <workbookView xWindow="15100" yWindow="680" windowWidth="15140" windowHeight="18980" activeTab="6" xr2:uid="{9C60B164-F6F9-DC45-9E1B-21FD8D75857B}"/>
   </bookViews>
   <sheets>
     <sheet name="MS4-3560" sheetId="1" r:id="rId1"/>
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="58" uniqueCount="17">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="109" uniqueCount="47">
   <si>
     <t>enable</t>
   </si>
@@ -93,6 +93,96 @@
   </si>
   <si>
     <t>show ipv6 general-prefix</t>
+  </si>
+  <si>
+    <t>vlan 10</t>
+  </si>
+  <si>
+    <t>name LAB1</t>
+  </si>
+  <si>
+    <t>vlan 20</t>
+  </si>
+  <si>
+    <t>name LAB2</t>
+  </si>
+  <si>
+    <t>vlan 30</t>
+  </si>
+  <si>
+    <t>name ADMIN</t>
+  </si>
+  <si>
+    <t>vlan 40</t>
+  </si>
+  <si>
+    <t>name ACADEMIC</t>
+  </si>
+  <si>
+    <t>vlan 50</t>
+  </si>
+  <si>
+    <t>name SERVER</t>
+  </si>
+  <si>
+    <t>exit</t>
+  </si>
+  <si>
+    <t>interface vlan 10</t>
+  </si>
+  <si>
+    <t>ipv6 address 2001:DB8:10::1/64</t>
+  </si>
+  <si>
+    <t>no shutdown</t>
+  </si>
+  <si>
+    <t>interface vlan 20</t>
+  </si>
+  <si>
+    <t>ipv6 address 2001:DB8:20::1/64</t>
+  </si>
+  <si>
+    <t>interface vlan 30</t>
+  </si>
+  <si>
+    <t>ipv6 address 2001:DB8:30::1/64</t>
+  </si>
+  <si>
+    <t>interface vlan 40</t>
+  </si>
+  <si>
+    <t>ipv6 address 2001:DB8:40::1/64</t>
+  </si>
+  <si>
+    <t>interface vlan 50</t>
+  </si>
+  <si>
+    <t>ipv6 address 2001:DB8:50::1/64</t>
+  </si>
+  <si>
+    <t>interface gi1/0/1</t>
+  </si>
+  <si>
+    <t>switchport mode trunk</t>
+  </si>
+  <si>
+    <t>interface gi1/0/2</t>
+  </si>
+  <si>
+    <t>interface gi1/0/4</t>
+  </si>
+  <si>
+    <t>interface gi1/0/3</t>
+  </si>
+  <si>
+    <t>no switchport</t>
+  </si>
+  <si>
+    <t>ipv6 address 2001:DB8:FF::1/64</t>
+  </si>
+  <si>
+    <t>ipv6 route ::/0 2001:DB8:FF::2</t>
   </si>
 </sst>
 </file>
@@ -171,12 +261,13 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -857,7 +948,7 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FD35A78F-566F-7848-A017-7C42AAF25B63}">
-  <dimension ref="A1:A8"/>
+  <dimension ref="A1:A77"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="46.6640625" customWidth="1"/>
@@ -901,6 +992,300 @@
     <row r="8" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A8" s="4" t="s">
         <v>7</v>
+      </c>
+    </row>
+    <row r="10" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A10" s="2" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A11" s="3" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="12" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A12" s="3" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="13" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A13" s="3" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="14" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A14" s="3" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="15" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A15" s="3" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="16" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A16" s="3" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="17" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A17" s="3" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="18" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A18" s="3" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="19" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A19" s="3" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="20" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A20" s="3" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="21" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A21" s="3" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="22" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A22" s="3"/>
+    </row>
+    <row r="23" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A23" s="3" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="24" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A24" s="3" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="25" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A25" s="3" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="26" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A26" s="4"/>
+    </row>
+    <row r="28" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A28" s="2" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="29" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A29" s="3" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="30" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A30" s="3" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="31" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A31" s="3" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="32" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A32" s="3" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="33" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A33" s="3"/>
+    </row>
+    <row r="34" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A34" s="3" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="35" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A35" s="3" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="36" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A36" s="3" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="37" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A37" s="3"/>
+    </row>
+    <row r="38" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A38" s="3" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="39" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A39" s="3" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="40" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A40" s="3" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="41" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A41" s="3"/>
+    </row>
+    <row r="42" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A42" s="3" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="43" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A43" s="3" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="44" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A44" s="3" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="45" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A45" s="3"/>
+    </row>
+    <row r="46" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A46" s="3" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="47" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A47" s="3" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="48" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A48" s="3" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="49" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A49" s="3"/>
+    </row>
+    <row r="50" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A50" s="4" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="52" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A52" s="2" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="53" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A53" s="3" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="54" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A54" s="3" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="55" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A55" s="3"/>
+    </row>
+    <row r="56" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A56" s="3" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="57" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A57" s="3" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="58" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A58" s="3" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="59" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A59" s="3"/>
+    </row>
+    <row r="60" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A60" s="3" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="61" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A61" s="3" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="62" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A62" s="3" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="63" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A63" s="3"/>
+    </row>
+    <row r="64" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A64" s="4" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="67" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A67" s="2" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="68" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A68" s="3" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="69" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A69" s="3" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="70" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A70" s="3" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="71" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A71" s="3"/>
+    </row>
+    <row r="72" spans="1:1" ht="17" x14ac:dyDescent="0.25">
+      <c r="A72" s="5" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="73" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A73" s="3" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="74" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A74" s="3"/>
+    </row>
+    <row r="75" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A75" s="3" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="76" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A76" s="3"/>
+    </row>
+    <row r="77" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A77" s="4" t="s">
+        <v>6</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
612 messages from MS2 fail
</commit_message>
<xml_diff>
--- a/2026-T1/T1B2-ICTNWK612-Plan-manage-troubleshooting-advance/2-tasks/script-PACKETTRACER.xlsx
+++ b/2026-T1/T1B2-ICTNWK612-Plan-manage-troubleshooting-advance/2-tasks/script-PACKETTRACER.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/mannsee/Documents/Assessments/2026-T1/T1B2-ICTNWK612-Plan-manage-troubleshooting-advance/2-tasks/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BB81FEE3-37C1-9241-998F-5F6F7D1ED8D1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E8EF6DF2-9DFA-BC4C-81F0-E4A8F986D944}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="15100" yWindow="680" windowWidth="15140" windowHeight="18980" activeTab="6" xr2:uid="{9C60B164-F6F9-DC45-9E1B-21FD8D75857B}"/>
+    <workbookView xWindow="16580" yWindow="660" windowWidth="13660" windowHeight="18980" firstSheet="2" activeTab="3" xr2:uid="{9C60B164-F6F9-DC45-9E1B-21FD8D75857B}"/>
   </bookViews>
   <sheets>
     <sheet name="MS4-3560" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,8 @@
     <sheet name="MS7-3560" sheetId="5" r:id="rId5"/>
     <sheet name="MS0-3650" sheetId="6" r:id="rId6"/>
     <sheet name="MS1-3650" sheetId="9" r:id="rId7"/>
-    <sheet name="CHECK-COMM" sheetId="10" r:id="rId8"/>
+    <sheet name="Firewall22" sheetId="11" r:id="rId8"/>
+    <sheet name="CHECK-COMM" sheetId="10" r:id="rId9"/>
   </sheets>
   <calcPr calcId="181029"/>
   <extLst>
@@ -42,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="109" uniqueCount="47">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="240" uniqueCount="69">
   <si>
     <t>enable</t>
   </si>
@@ -183,13 +184,79 @@
   </si>
   <si>
     <t>ipv6 route ::/0 2001:DB8:FF::2</t>
+  </si>
+  <si>
+    <t>interface gi0/1</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> no shutdown</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> switchport mode access</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> switchport access vlan 10</t>
+  </si>
+  <si>
+    <t>erase startup-config</t>
+  </si>
+  <si>
+    <t>interface range fa0/1-24</t>
+  </si>
+  <si>
+    <t>switchport trunk encapsulation dot1q</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> switchport access vlan 30</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> switchport access vlan 20</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> switchport access vlan 40</t>
+  </si>
+  <si>
+    <t>hostname Firewall22</t>
+  </si>
+  <si>
+    <t>interface GigabitEthernet1/2</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> nameif inside</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> security-level 100</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> ipv6 address 2001:DB8:FF::2/64</t>
+  </si>
+  <si>
+    <t>interface GigabitEthernet1/1</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> nameif outside</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> security-level 0</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> ipv6 address 2001:DB8:100::1/64</t>
+  </si>
+  <si>
+    <t>ipv6 route inside 2001:DB8::/32 2001:DB8:FF::1</t>
+  </si>
+  <si>
+    <t>ipv6 route outside ::/0 2001:DB8:100::2</t>
+  </si>
+  <si>
+    <t>ipv6 address 2001:DB8:100::2/64</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -203,13 +270,26 @@
       <name val="Arial Unicode MS"/>
       <family val="2"/>
     </font>
+    <font>
+      <sz val="12"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="4">
@@ -261,13 +341,20 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -582,7 +669,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B34311B4-1E30-6D40-A73D-B4C7308E242A}">
-  <dimension ref="A1:A23"/>
+  <dimension ref="A1:A33"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="54.83203125" customWidth="1"/>
@@ -605,37 +692,133 @@
     </row>
     <row r="4" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A4" s="3" t="s">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="5" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A5" s="3" t="s">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="6" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A6" s="3" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
     </row>
     <row r="7" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A7" s="3" t="s">
+      <c r="A7" s="4" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="10" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A10" s="2" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A11" s="3" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="12" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A12" s="3" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="13" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A13" s="3" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="14" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A14" s="3" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="15" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A15" s="3" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="16" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A16" s="3" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="17" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A17" s="3"/>
+    </row>
+    <row r="18" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A18" s="3" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="19" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A19" s="3"/>
+    </row>
+    <row r="20" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A20" s="3" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="21" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A21" s="3" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="22" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A22" s="3" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="23" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A23" s="3" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="24" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A24" s="3" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="25" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A25" s="3"/>
+    </row>
+    <row r="26" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A26" s="3" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="27" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A27" s="3" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="28" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A28" s="3" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="29" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A29" s="3"/>
+    </row>
+    <row r="30" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A30" s="3" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="31" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A31" s="3"/>
+    </row>
+    <row r="32" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A32" s="3" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="33" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A33" s="4" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="8" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A8" s="4" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="11" spans="1:1" ht="17" x14ac:dyDescent="0.25">
-      <c r="A11" s="1"/>
-    </row>
-    <row r="22" spans="1:1" ht="17" x14ac:dyDescent="0.25">
-      <c r="A22" s="1"/>
-    </row>
-    <row r="23" spans="1:1" ht="17" x14ac:dyDescent="0.25">
-      <c r="A23" s="1"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -644,7 +827,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{59A2DE29-DDFD-084F-996E-5D8DD645CFD2}">
-  <dimension ref="A1:A8"/>
+  <dimension ref="A1:A33"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="34.1640625" customWidth="1"/>
@@ -667,27 +850,132 @@
     </row>
     <row r="4" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A4" s="3" t="s">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="5" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A5" s="3" t="s">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="6" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A6" s="3" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
     </row>
     <row r="7" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A7" s="3" t="s">
+      <c r="A7" s="4" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="10" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A10" s="7" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A11" s="6" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="12" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A12" s="6" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="13" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A13" s="6" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="14" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A14" s="6" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="15" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A15" s="6" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="16" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A16" s="6" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="17" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A17" s="6"/>
+    </row>
+    <row r="18" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A18" s="6" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="19" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A19" s="6"/>
+    </row>
+    <row r="20" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A20" s="6" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="21" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A21" s="6" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="22" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A22" s="6" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="23" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A23" s="6" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="24" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A24" s="6" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="25" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A25" s="6"/>
+    </row>
+    <row r="26" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A26" s="6" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="27" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A27" s="6" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="28" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A28" s="6" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="29" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A29" s="6"/>
+    </row>
+    <row r="30" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A30" s="6" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="31" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A31" s="6"/>
+    </row>
+    <row r="32" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A32" s="6" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="33" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A33" s="8" t="s">
         <v>6</v>
-      </c>
-    </row>
-    <row r="8" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A8" s="4" t="s">
-        <v>7</v>
       </c>
     </row>
   </sheetData>
@@ -697,7 +985,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CCC59594-6BB4-1E4A-B489-1D5AC66DAC96}">
-  <dimension ref="A1:A8"/>
+  <dimension ref="A1:A32"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="43.83203125" customWidth="1"/>
@@ -720,27 +1008,132 @@
     </row>
     <row r="4" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A4" s="3" t="s">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="5" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A5" s="3" t="s">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="6" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A6" s="3" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
     </row>
     <row r="7" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A7" s="3" t="s">
+      <c r="A7" s="4" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="9" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A9" s="2" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="10" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A10" s="3" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="11" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A11" s="3" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="12" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A12" s="3" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="13" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A13" s="3" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="14" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A14" s="3" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="15" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A15" s="3" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="16" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A16" s="3"/>
+    </row>
+    <row r="17" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A17" s="3" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="18" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A18" s="3"/>
+    </row>
+    <row r="19" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A19" s="3" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="20" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A20" s="3" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="21" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A21" s="3" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="22" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A22" s="3" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="23" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A23" s="3" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="24" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A24" s="3"/>
+    </row>
+    <row r="25" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A25" s="3" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="26" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A26" s="3" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="27" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A27" s="3" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="28" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A28" s="3"/>
+    </row>
+    <row r="29" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A29" s="3" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="30" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A30" s="3"/>
+    </row>
+    <row r="31" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A31" s="3" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="32" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A32" s="4" t="s">
         <v>6</v>
-      </c>
-    </row>
-    <row r="8" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A8" s="4" t="s">
-        <v>7</v>
       </c>
     </row>
   </sheetData>
@@ -750,10 +1143,10 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B10D8871-2FF1-AB46-91D6-9529E44202B6}">
-  <dimension ref="A1:A8"/>
+  <dimension ref="A1:A29"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="32.83203125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="56.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.2">
@@ -773,12 +1166,12 @@
     </row>
     <row r="4" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A4" s="3" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="5" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A5" t="s">
         <v>3</v>
-      </c>
-    </row>
-    <row r="5" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A5" s="3" t="s">
-        <v>4</v>
       </c>
     </row>
     <row r="6" spans="1:1" x14ac:dyDescent="0.2">
@@ -794,6 +1187,93 @@
     <row r="8" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A8" s="4" t="s">
         <v>7</v>
+      </c>
+    </row>
+    <row r="11" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A11" s="9" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="12" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A12" s="10" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="13" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A13" s="10" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="14" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A14" s="10" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="15" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A15" s="10" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="16" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A16" s="10" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="17" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A17" s="10" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="18" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A18" s="10"/>
+    </row>
+    <row r="19" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A19" s="10" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="20" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A20" s="10"/>
+    </row>
+    <row r="21" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A21" s="11" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="22" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A22" s="11" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="23" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A23" s="11" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="24" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A24" s="11" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="25" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A25" s="10"/>
+    </row>
+    <row r="26" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A26" s="10" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="27" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A27" s="10"/>
+    </row>
+    <row r="28" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A28" s="10" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="29" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A29" s="12" t="s">
+        <v>6</v>
       </c>
     </row>
   </sheetData>
@@ -803,7 +1283,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{48880218-5589-A547-BB90-D873A156AAD1}">
-  <dimension ref="A1:A29"/>
+  <dimension ref="A1:A33"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="52.5" customWidth="1"/>
@@ -826,67 +1306,133 @@
     </row>
     <row r="4" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A4" s="3" t="s">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="5" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A5" s="3" t="s">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="6" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A6" s="3" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
     </row>
     <row r="7" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A7" s="3" t="s">
+      <c r="A7" s="4" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="10" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A10" s="7" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A11" s="6" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="12" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A12" s="6" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="13" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A13" s="6" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="14" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A14" s="6" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="15" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A15" s="6" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="16" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A16" s="6" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="17" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A17" s="6"/>
+    </row>
+    <row r="18" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A18" s="6" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="19" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A19" s="6"/>
+    </row>
+    <row r="20" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A20" s="6" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="21" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A21" s="6" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="22" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A22" s="6" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="23" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A23" s="6" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="24" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A24" s="6" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="25" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A25" s="6"/>
+    </row>
+    <row r="26" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A26" s="6" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="27" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A27" s="6" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="28" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A28" s="6" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="29" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A29" s="6"/>
+    </row>
+    <row r="30" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A30" s="6" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="31" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A31" s="6"/>
+    </row>
+    <row r="32" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A32" s="6" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="33" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A33" s="8" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="8" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A8" s="4" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="12" spans="1:1" ht="17" x14ac:dyDescent="0.25">
-      <c r="A12" s="1"/>
-    </row>
-    <row r="14" spans="1:1" ht="17" x14ac:dyDescent="0.25">
-      <c r="A14" s="1"/>
-    </row>
-    <row r="15" spans="1:1" ht="17" x14ac:dyDescent="0.25">
-      <c r="A15" s="1"/>
-    </row>
-    <row r="17" spans="1:1" ht="17" x14ac:dyDescent="0.25">
-      <c r="A17" s="1"/>
-    </row>
-    <row r="18" spans="1:1" ht="17" x14ac:dyDescent="0.25">
-      <c r="A18" s="1"/>
-    </row>
-    <row r="19" spans="1:1" ht="17" x14ac:dyDescent="0.25">
-      <c r="A19" s="1"/>
-    </row>
-    <row r="20" spans="1:1" ht="17" x14ac:dyDescent="0.25">
-      <c r="A20" s="1"/>
-    </row>
-    <row r="22" spans="1:1" ht="17" x14ac:dyDescent="0.25">
-      <c r="A22" s="1"/>
-    </row>
-    <row r="23" spans="1:1" ht="17" x14ac:dyDescent="0.25">
-      <c r="A23" s="1"/>
-    </row>
-    <row r="24" spans="1:1" ht="17" x14ac:dyDescent="0.25">
-      <c r="A24" s="1"/>
-    </row>
-    <row r="26" spans="1:1" ht="17" x14ac:dyDescent="0.25">
-      <c r="A26" s="1"/>
-    </row>
-    <row r="27" spans="1:1" ht="17" x14ac:dyDescent="0.25">
-      <c r="A27" s="1"/>
-    </row>
-    <row r="29" spans="1:1" ht="17" x14ac:dyDescent="0.25">
-      <c r="A29" s="1"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -895,7 +1441,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6CFEE1F6-6AF7-454F-BBB3-C95B039FA8B6}">
-  <dimension ref="A1:A8"/>
+  <dimension ref="A1:A37"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="36" customWidth="1"/>
@@ -918,27 +1464,148 @@
     </row>
     <row r="4" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A4" s="3" t="s">
-        <v>13</v>
+        <v>4</v>
       </c>
     </row>
     <row r="5" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A5" s="3" t="s">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="6" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A6" s="3" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
     </row>
     <row r="7" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A7" s="3" t="s">
+      <c r="A7" s="4" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="10" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A10" s="2" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A11" s="3" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="12" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A12" s="3" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="13" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A13" s="3" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="14" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A14" s="3" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="15" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A15" s="3" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="16" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A16" s="3" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="17" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A17" s="3"/>
+    </row>
+    <row r="18" spans="1:1" ht="17" x14ac:dyDescent="0.25">
+      <c r="A18" s="5" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="19" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A19" s="3"/>
+    </row>
+    <row r="20" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A20" s="3" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="21" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A21" s="3" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="22" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A22" s="3" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="23" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A23" s="3"/>
+    </row>
+    <row r="24" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A24" s="3" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="25" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A25" s="3"/>
+    </row>
+    <row r="26" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A26" s="3" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="27" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A27" s="3" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="28" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A28" s="3" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="29" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A29" s="3"/>
+    </row>
+    <row r="30" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A30" s="3" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="31" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A31" s="3" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="32" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A32" s="3" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="33" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A33" s="3"/>
+    </row>
+    <row r="34" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A34" s="3" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="35" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A35" s="3"/>
+    </row>
+    <row r="36" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A36" s="3" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="37" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A37" s="4" t="s">
         <v>6</v>
-      </c>
-    </row>
-    <row r="8" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A8" s="4" t="s">
-        <v>7</v>
       </c>
     </row>
   </sheetData>
@@ -948,7 +1615,7 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FD35A78F-566F-7848-A017-7C42AAF25B63}">
-  <dimension ref="A1:A77"/>
+  <dimension ref="A1:A74"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="46.6640625" customWidth="1"/>
@@ -1273,18 +1940,7 @@
       </c>
     </row>
     <row r="74" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A74" s="3"/>
-    </row>
-    <row r="75" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A75" s="3" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="76" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A76" s="3"/>
-    </row>
-    <row r="77" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A77" s="4" t="s">
+      <c r="A74" s="4" t="s">
         <v>6</v>
       </c>
     </row>
@@ -1294,9 +1950,163 @@
 </file>
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4B6DA10D-BF52-0741-AE7A-9E4881301AC3}">
+  <dimension ref="A1:A31"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="1" max="1" width="45" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A1" s="2" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="2" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A2" s="3" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A3" s="3" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="4" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A4" s="3" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="5" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A5" s="3" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="6" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A6" s="4" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="8" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A8" s="2" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A9" s="3" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="10" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A10" s="3" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="11" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A11" s="3" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="12" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A12" s="3" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="13" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A13" s="3" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="14" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A14" s="3" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="15" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A15" s="3"/>
+    </row>
+    <row r="16" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A16" s="3" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="17" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A17" s="3"/>
+    </row>
+    <row r="18" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A18" s="3" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="19" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A19" s="3" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="20" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A20" s="3" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="21" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A21" s="3" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="22" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A22" s="3" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="23" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A23" s="3"/>
+    </row>
+    <row r="24" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A24" s="3" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="25" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A25" s="3"/>
+    </row>
+    <row r="26" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A26" s="3" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="27" spans="1:1" ht="17" x14ac:dyDescent="0.25">
+      <c r="A27" s="5" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="28" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A28" s="3"/>
+    </row>
+    <row r="29" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A29" s="3" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="30" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A30" s="3"/>
+    </row>
+    <row r="31" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A31" s="4" t="s">
+        <v>6</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E50F22F7-84B5-DE40-B8F5-33EE5991EA40}">
-  <dimension ref="A1:A2"/>
+  <dimension ref="A1:A21"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="1" max="1" width="52.6640625" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
@@ -1308,6 +2118,11 @@
         <v>16</v>
       </c>
     </row>
+    <row r="21" spans="1:1" ht="17" x14ac:dyDescent="0.25">
+      <c r="A21" s="1" t="s">
+        <v>51</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
612 before ASA config Access control list
</commit_message>
<xml_diff>
--- a/2026-T1/T1B2-ICTNWK612-Plan-manage-troubleshooting-advance/2-tasks/script-PACKETTRACER.xlsx
+++ b/2026-T1/T1B2-ICTNWK612-Plan-manage-troubleshooting-advance/2-tasks/script-PACKETTRACER.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10222"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10302"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/mannsee/Documents/Assessments/2026-T1/T1B2-ICTNWK612-Plan-manage-troubleshooting-advance/2-tasks/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E8EF6DF2-9DFA-BC4C-81F0-E4A8F986D944}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{18B63D02-1C92-1A4E-A517-6D67E1F1C59F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="16580" yWindow="660" windowWidth="13660" windowHeight="18980" firstSheet="2" activeTab="3" xr2:uid="{9C60B164-F6F9-DC45-9E1B-21FD8D75857B}"/>
+    <workbookView xWindow="16580" yWindow="660" windowWidth="13660" windowHeight="18980" activeTab="3" xr2:uid="{9C60B164-F6F9-DC45-9E1B-21FD8D75857B}"/>
   </bookViews>
   <sheets>
     <sheet name="MS4-3560" sheetId="1" r:id="rId1"/>
@@ -43,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="240" uniqueCount="69">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="260" uniqueCount="77">
   <si>
     <t>enable</t>
   </si>
@@ -250,6 +250,30 @@
   </si>
   <si>
     <t>ipv6 address 2001:DB8:100::2/64</t>
+  </si>
+  <si>
+    <t>policy-map global_policy</t>
+  </si>
+  <si>
+    <t>inspect icmp error</t>
+  </si>
+  <si>
+    <t>inspect icmp</t>
+  </si>
+  <si>
+    <t>class inspection_default</t>
+  </si>
+  <si>
+    <t>end</t>
+  </si>
+  <si>
+    <t>ipv6 route ::/0 2001:DB8:100::1</t>
+  </si>
+  <si>
+    <t>switchport mode access</t>
+  </si>
+  <si>
+    <t>switchport access vlan 50</t>
   </si>
 </sst>
 </file>
@@ -1143,7 +1167,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B10D8871-2FF1-AB46-91D6-9529E44202B6}">
-  <dimension ref="A1:A29"/>
+  <dimension ref="A1:A49"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="56.83203125" customWidth="1"/>
@@ -1175,92 +1199,94 @@
       </c>
     </row>
     <row r="6" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A6" s="3" t="s">
-        <v>5</v>
+      <c r="A6" t="s">
+        <v>13</v>
       </c>
     </row>
     <row r="7" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A7" s="3" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="8" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A8" s="3" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="8" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A8" s="4" t="s">
+    <row r="9" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A9" s="4" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="11" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A11" s="9" t="s">
+    <row r="12" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A12" s="9" t="s">
         <v>0</v>
-      </c>
-    </row>
-    <row r="12" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A12" s="10" t="s">
-        <v>1</v>
       </c>
     </row>
     <row r="13" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A13" s="10" t="s">
-        <v>17</v>
+        <v>1</v>
       </c>
     </row>
     <row r="14" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A14" s="10" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
     </row>
     <row r="15" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A15" s="10" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
     </row>
     <row r="16" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A16" s="10" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
     </row>
     <row r="17" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A17" s="10" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="18" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A18" s="3" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="18" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A18" s="10"/>
-    </row>
     <row r="19" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A19" s="10" t="s">
-        <v>27</v>
+      <c r="A19" s="3" t="s">
+        <v>26</v>
       </c>
     </row>
     <row r="20" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A20" s="10"/>
+      <c r="A20" s="3"/>
     </row>
     <row r="21" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A21" s="11" t="s">
-        <v>47</v>
+      <c r="A21" s="10" t="s">
+        <v>27</v>
       </c>
     </row>
     <row r="22" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A22" s="11" t="s">
-        <v>44</v>
-      </c>
+      <c r="A22" s="10"/>
     </row>
     <row r="23" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A23" s="11" t="s">
-        <v>68</v>
+        <v>47</v>
       </c>
     </row>
     <row r="24" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A24" s="11" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="25" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A25" s="11" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="26" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A26" s="11" t="s">
         <v>30</v>
-      </c>
-    </row>
-    <row r="25" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A25" s="10"/>
-    </row>
-    <row r="26" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A26" s="10" t="s">
-        <v>27</v>
       </c>
     </row>
     <row r="27" spans="1:1" x14ac:dyDescent="0.2">
@@ -1272,7 +1298,65 @@
       </c>
     </row>
     <row r="29" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A29" s="12" t="s">
+      <c r="A29" s="10"/>
+    </row>
+    <row r="30" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A30" s="10" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="31" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A31" s="12" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="34" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A34" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="35" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A35" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="36" spans="1:1" ht="17" x14ac:dyDescent="0.25">
+      <c r="A36" s="1" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="41" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A41" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="42" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A42" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="43" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A43" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="44" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A44" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="46" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A46" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="47" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A47" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="49" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A49" t="s">
         <v>6</v>
       </c>
     </row>
@@ -1951,7 +2035,7 @@
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4B6DA10D-BF52-0741-AE7A-9E4881301AC3}">
-  <dimension ref="A1:A31"/>
+  <dimension ref="A1:A41"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="45" customWidth="1"/>
@@ -2092,6 +2176,46 @@
     </row>
     <row r="31" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A31" s="4" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="34" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A34" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="35" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A35" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="36" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A36" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="37" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A37" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="38" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A38" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="39" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A39" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="40" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A40" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="41" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A41" t="s">
         <v>6</v>
       </c>
     </row>

</xml_diff>